<commit_message>
forex + quant risk mgmt
</commit_message>
<xml_diff>
--- a/group-project/group-project-rubric.xlsx
+++ b/group-project/group-project-rubric.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/T7/Dropbox/LBS/01_websites_github_repos/e628-shared/group-project/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{160B0ED0-4156-B14B-9AD1-9D699EDB4155}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D175E96A-AAAC-6B40-8580-6B5F8E39D191}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="67200" windowHeight="35520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1540,7 +1540,7 @@
       </c>
       <c r="D46" s="4"/>
     </row>
-    <row r="47" spans="1:4" ht="80" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:4" ht="128" x14ac:dyDescent="0.2">
       <c r="A47" s="20"/>
       <c r="B47" s="20"/>
       <c r="C47" s="5" t="s">

</xml_diff>